<commit_message>
Add per-job monthly revenue table (2026 Jan-May)
New "Job Revenue 2026" sheet + data/Job_Revenue_2026_byMonth.csv: all 140 jobs
with revenue billed in 2026, broken out by month (Jan-May) with a Jan-May total,
sorted largest first. Source = Knowify InvoicesSummaryReport (269 invoices, by
invoice date); grand total $20.28M. build_excel.py renders the sheet when the
CSV is present, so it survives refreshes.

https://claude.ai/code/session_01CqWT8xJUtGR2BEPYF4o2h5
</commit_message>
<xml_diff>
--- a/mdg-powerbi/output/MDG_Executive_Dashboard.xlsx
+++ b/mdg-powerbi/output/MDG_Executive_Dashboard.xlsx
@@ -30,6 +30,7 @@
     <sheet name="» Dim_Division" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="» Dim_PM" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="» Param_Cash" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Job Revenue 2026" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70531,6 +70532,3619 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000F1F3D"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N145"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Revenue Billed by Job — 2026 (Jan–May)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Knowify invoices by invoice date  •  140 jobs with 2026 revenue  •  sorted largest first</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>Total Jan-May</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>MF.2025.972 Union Flats - Fishers</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="n">
+        <v>27090</v>
+      </c>
+      <c r="C5" s="18" t="n">
+        <v>229770</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>486459</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>841491</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>571623.75</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>2156433.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>MF.2025.1019 Town &amp; Country Apartments (NY MF Project - 22 bldgs)</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>246097.48</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>562089.22</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>675814.0699999999</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>435716.98</v>
+      </c>
+      <c r="G6" s="35" t="n">
+        <v>1919717.75</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>2025.964 Avon Municipal Building</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>363417.48</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>173192.63</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>226932.38</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>220010.73</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>236453.93</v>
+      </c>
+      <c r="G7" s="35" t="n">
+        <v>1220007.15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>MF.2024.931 Wild Air</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>166011.35</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>148756.83</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>226412.55</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>408053.89</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>126290.65</v>
+      </c>
+      <c r="G8" s="35" t="n">
+        <v>1075525.27</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>2025.1029 Resmed - Indy 500</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>41976.09</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>65098.75</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>104940.22</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>538961.21</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>217317.46</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>968293.73</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>MF.2025.989-2 Springdale Cinema - Drywall</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>122512.5</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>224842.5</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>256635</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>344520</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>948510</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>2025.1024 Metro Lion</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>231487.2</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>553922.8</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F11" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="35" t="n">
+        <v>786710</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>2025.991 Walmart Republic</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="n">
+        <v>65246.93</v>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>194391.63</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>141074.42</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>186798.6</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="35" t="n">
+        <v>587511.58</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>2025.978 Ardalan Plaza</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>29270.16</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>88455.24000000001</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>182393.32</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>58873.86</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <v>193598.5</v>
+      </c>
+      <c r="G13" s="35" t="n">
+        <v>552591.08</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>MF.2024.928 Holliday Farms Assisted Living - Zionsville</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>75888.38</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>23629.34</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>56885.34</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>54038.62</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>338327.69</v>
+      </c>
+      <c r="G14" s="35" t="n">
+        <v>548769.37</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>2025.1001 Evolve Transporters</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>290318.22</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>204675.12</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>10660.05</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>30489.3</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>1341</v>
+      </c>
+      <c r="G15" s="35" t="n">
+        <v>537483.6899999999</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>2025.1023 Vikan Products BTS</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>16087.5</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>95690.7</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>205262.77</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>198556.32</v>
+      </c>
+      <c r="G16" s="35" t="n">
+        <v>515597.29</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>2025.1030 Westfield Police HQ</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>94815</v>
+      </c>
+      <c r="F17" s="18" t="n">
+        <v>420570</v>
+      </c>
+      <c r="G17" s="35" t="n">
+        <v>515385</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>MF.2024.892 The Lofts at Headwaters Park</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n">
+        <v>161432.46</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>114855.12</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>62543.7</v>
+      </c>
+      <c r="E18" s="18" t="n">
+        <v>89590.28</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>63353.47</v>
+      </c>
+      <c r="G18" s="35" t="n">
+        <v>491775.03</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>2025.990 Walmart Orlando</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="n">
+        <v>55072.44</v>
+      </c>
+      <c r="C19" s="18" t="n">
+        <v>100249.47</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <v>127771.38</v>
+      </c>
+      <c r="E19" s="18" t="n">
+        <v>133941.78</v>
+      </c>
+      <c r="F19" s="18" t="n">
+        <v>74099.78999999999</v>
+      </c>
+      <c r="G19" s="35" t="n">
+        <v>491134.86</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>MF.2025.992 Young's Creek Apartments</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="n">
+        <v>127149.57</v>
+      </c>
+      <c r="C20" s="18" t="n">
+        <v>58491.67</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>30618</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>272493.11</v>
+      </c>
+      <c r="F20" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="35" t="n">
+        <v>488752.35</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>2026.1035 The Ark</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="18" t="n">
+        <v>228065.58</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>86809.67999999999</v>
+      </c>
+      <c r="F21" s="18" t="n">
+        <v>156749.71</v>
+      </c>
+      <c r="G21" s="35" t="n">
+        <v>471624.97</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>MF.2025.989-1 Springdale Cinema - Paint</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="18" t="n">
+        <v>55440</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>165847.5</v>
+      </c>
+      <c r="F22" s="18" t="n">
+        <v>206955</v>
+      </c>
+      <c r="G22" s="35" t="n">
+        <v>428242.5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Priority Way Office</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="18" t="n">
+        <v>413250</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="35" t="n">
+        <v>413250</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>2025.1026 HNTB Buildout (Salesforce Tower)</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="n">
+        <v>40056.3</v>
+      </c>
+      <c r="C24" s="18" t="n">
+        <v>92546.64</v>
+      </c>
+      <c r="D24" s="18" t="n">
+        <v>111708.94</v>
+      </c>
+      <c r="E24" s="18" t="n">
+        <v>75748.67999999999</v>
+      </c>
+      <c r="F24" s="18" t="n">
+        <v>92235.03999999999</v>
+      </c>
+      <c r="G24" s="35" t="n">
+        <v>412295.6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>2026.1042 SND2 at ILP Bldg IV Whitestown</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>164669.04</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>68841.53999999999</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>123216.76</v>
+      </c>
+      <c r="G25" s="35" t="n">
+        <v>356727.34</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>MF.2024.945 Encore Senior Living</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="n">
+        <v>43797.38</v>
+      </c>
+      <c r="C26" s="18" t="n">
+        <v>94697.22</v>
+      </c>
+      <c r="D26" s="18" t="n">
+        <v>54087.55</v>
+      </c>
+      <c r="E26" s="18" t="n">
+        <v>91941.31</v>
+      </c>
+      <c r="F26" s="18" t="n">
+        <v>61193.27</v>
+      </c>
+      <c r="G26" s="35" t="n">
+        <v>345716.73</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>2024.950 Caterpillar Triple Crown</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="n">
+        <v>9448.35</v>
+      </c>
+      <c r="C27" s="18" t="n">
+        <v>147545.92</v>
+      </c>
+      <c r="D27" s="18" t="n">
+        <v>38045.07</v>
+      </c>
+      <c r="E27" s="18" t="n">
+        <v>72880.67</v>
+      </c>
+      <c r="F27" s="18" t="n">
+        <v>36620.15</v>
+      </c>
+      <c r="G27" s="35" t="n">
+        <v>304540.16</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>2025.994 Stotan Port Laredo Spec Offices</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="n">
+        <v>107527.5</v>
+      </c>
+      <c r="C28" s="18" t="n">
+        <v>25920</v>
+      </c>
+      <c r="D28" s="18" t="n">
+        <v>27180</v>
+      </c>
+      <c r="E28" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="18" t="n">
+        <v>114932.8</v>
+      </c>
+      <c r="G28" s="35" t="n">
+        <v>275560.3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>MF.2026.1050 AC Hotel</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="18" t="n">
+        <v>202650.67</v>
+      </c>
+      <c r="G29" s="35" t="n">
+        <v>202650.67</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>2026.1033 Avon Demising Wall</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="18" t="n">
+        <v>181500</v>
+      </c>
+      <c r="E30" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="35" t="n">
+        <v>181500</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>2024.909 Andretti Global HQ</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="n">
+        <v>40682</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="18" t="n">
+        <v>129947</v>
+      </c>
+      <c r="G31" s="35" t="n">
+        <v>170629</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>2026.1038 Artistic Composite Pallet Expansion</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="18" t="n">
+        <v>104592.42</v>
+      </c>
+      <c r="E32" s="18" t="n">
+        <v>65920.59</v>
+      </c>
+      <c r="F32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="35" t="n">
+        <v>170513.01</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>2025.1006 Keller Office</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="18" t="n">
+        <v>168520.5</v>
+      </c>
+      <c r="G33" s="35" t="n">
+        <v>168520.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>2026.1041 Whiteland Building 2 - Blackhawk</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="18" t="n">
+        <v>111888</v>
+      </c>
+      <c r="F34" s="18" t="n">
+        <v>44532.3</v>
+      </c>
+      <c r="G34" s="35" t="n">
+        <v>156420.3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>2026.1047 Springdale Building 4 Demising Walls</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="18" t="n">
+        <v>148800</v>
+      </c>
+      <c r="G35" s="35" t="n">
+        <v>148800</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>2025.1027 Indy Boat Co</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="18" t="n">
+        <v>53062.2</v>
+      </c>
+      <c r="F36" s="18" t="n">
+        <v>83283.7</v>
+      </c>
+      <c r="G36" s="35" t="n">
+        <v>136345.9</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>2026.1043 Deer Creek Building 1</t>
+        </is>
+      </c>
+      <c r="B37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="18" t="n">
+        <v>135000</v>
+      </c>
+      <c r="E37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="35" t="n">
+        <v>135000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>2026.1045 First OnSite (Ameriplex)</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="18" t="n">
+        <v>128000</v>
+      </c>
+      <c r="F38" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="35" t="n">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>2026.1037 CV - Castle Rock</t>
+        </is>
+      </c>
+      <c r="B39" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="18" t="n">
+        <v>125451</v>
+      </c>
+      <c r="D39" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G39" s="35" t="n">
+        <v>127451</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>2026.1046 Automatic Distributors (Park 130 Bldg 6)</t>
+        </is>
+      </c>
+      <c r="B40" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="18" t="n">
+        <v>32697</v>
+      </c>
+      <c r="F40" s="18" t="n">
+        <v>91953</v>
+      </c>
+      <c r="G40" s="35" t="n">
+        <v>124650</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>2025.967 Bunge Project Flex</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="18" t="n">
+        <v>11965.23</v>
+      </c>
+      <c r="D41" s="18" t="n">
+        <v>109085.8</v>
+      </c>
+      <c r="E41" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="35" t="n">
+        <v>121051.03</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>2026.1036 Port Laredo Trade Center</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="18" t="n">
+        <v>73818</v>
+      </c>
+      <c r="E42" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="18" t="n">
+        <v>34657</v>
+      </c>
+      <c r="G42" s="35" t="n">
+        <v>108475</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>2025.1012 Airport South Logistics Bldg. B</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="18" t="n">
+        <v>9868.5</v>
+      </c>
+      <c r="E43" s="18" t="n">
+        <v>26117.77</v>
+      </c>
+      <c r="F43" s="18" t="n">
+        <v>67259.03</v>
+      </c>
+      <c r="G43" s="35" t="n">
+        <v>103245.3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>MF.2025.977 Civic Square Condos</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="n">
+        <v>16373.48</v>
+      </c>
+      <c r="C44" s="18" t="n">
+        <v>2902.5</v>
+      </c>
+      <c r="D44" s="18" t="n">
+        <v>3275.1</v>
+      </c>
+      <c r="E44" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="18" t="n">
+        <v>61611.56</v>
+      </c>
+      <c r="G44" s="35" t="n">
+        <v>84162.64</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>MF.2025.975 The Eleven - Monon Square</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="18" t="n">
+        <v>30587.39</v>
+      </c>
+      <c r="F45" s="18" t="n">
+        <v>47118.33</v>
+      </c>
+      <c r="G45" s="35" t="n">
+        <v>77705.72</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>2025.1032 65 Commerce Park Building 7</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="18" t="n">
+        <v>71314.2</v>
+      </c>
+      <c r="G46" s="35" t="n">
+        <v>71314.2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>2025.981 Fort Ben - Foamcraft</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="18" t="n">
+        <v>69374.88</v>
+      </c>
+      <c r="D47" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="35" t="n">
+        <v>69374.88</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>MF.2025.976 Firefly Youth Housing</t>
+        </is>
+      </c>
+      <c r="B48" s="18" t="n">
+        <v>4050</v>
+      </c>
+      <c r="C48" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="18" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E48" s="18" t="n">
+        <v>36934.63</v>
+      </c>
+      <c r="F48" s="18" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G48" s="35" t="n">
+        <v>67984.63</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>2023.839 Hamilton County National Guard Readiness Center</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="18" t="n">
+        <v>58016.76</v>
+      </c>
+      <c r="F49" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="35" t="n">
+        <v>58016.76</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>2025.1015 WBP Lot 4</t>
+        </is>
+      </c>
+      <c r="B50" s="18" t="n">
+        <v>31758.75</v>
+      </c>
+      <c r="C50" s="18" t="n">
+        <v>18902.5</v>
+      </c>
+      <c r="D50" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="18" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F50" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="35" t="n">
+        <v>56161.25</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>2025.966 C5 Bullitt III Logistics Center Warehouse</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="n">
+        <v>56050.1</v>
+      </c>
+      <c r="C51" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="35" t="n">
+        <v>56050.1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>2026.1034 Stella's Ice Cream Shop</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="18" t="n">
+        <v>22860</v>
+      </c>
+      <c r="E52" s="18" t="n">
+        <v>11250</v>
+      </c>
+      <c r="F52" s="18" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G52" s="35" t="n">
+        <v>52110</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>2025.1016 WBP Lot C</t>
+        </is>
+      </c>
+      <c r="B53" s="18" t="n">
+        <v>25903.13</v>
+      </c>
+      <c r="C53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="18" t="n">
+        <v>13081.87</v>
+      </c>
+      <c r="G53" s="35" t="n">
+        <v>38985</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>2025.979 Groundbreakers</t>
+        </is>
+      </c>
+      <c r="B54" s="18" t="n">
+        <v>5282.37</v>
+      </c>
+      <c r="C54" s="18" t="n">
+        <v>32067.74</v>
+      </c>
+      <c r="D54" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="35" t="n">
+        <v>37350.11</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>2025.1013 Lucas Oil Corydon</t>
+        </is>
+      </c>
+      <c r="B55" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="18" t="n">
+        <v>22500</v>
+      </c>
+      <c r="D55" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="18" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G55" s="35" t="n">
+        <v>32500</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>2024.913 Walmart Phoenix</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="18" t="n">
+        <v>25857</v>
+      </c>
+      <c r="E56" s="18" t="n">
+        <v>3055.5</v>
+      </c>
+      <c r="F56" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="35" t="n">
+        <v>28912.5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>2023.843 Walmart Frederick</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="18" t="n">
+        <v>26200</v>
+      </c>
+      <c r="E57" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="35" t="n">
+        <v>26200</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2404 Flores Sandhu Res</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="18" t="n">
+        <v>20852.65</v>
+      </c>
+      <c r="E58" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="35" t="n">
+        <v>20852.65</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>2026.1056 Senator Banks Office</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="18" t="n">
+        <v>20467.33</v>
+      </c>
+      <c r="G59" s="35" t="n">
+        <v>20467.33</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2387 0204 Jose Irachetta</t>
+        </is>
+      </c>
+      <c r="B60" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C60" s="18" t="n">
+        <v>20097.86</v>
+      </c>
+      <c r="D60" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="35" t="n">
+        <v>20097.86</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>2025.1025 Park 100 - Building 22</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="n">
+        <v>19640</v>
+      </c>
+      <c r="C61" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="35" t="n">
+        <v>19640</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2376 5724 E Southport Rd</t>
+        </is>
+      </c>
+      <c r="B62" s="18" t="n">
+        <v>18119.63</v>
+      </c>
+      <c r="C62" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="35" t="n">
+        <v>18119.63</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>2025.1028 Northpoint</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="18" t="n">
+        <v>17415</v>
+      </c>
+      <c r="F63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="35" t="n">
+        <v>17415</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>2025.993 Batesville Public Library</t>
+        </is>
+      </c>
+      <c r="B64" s="18" t="n">
+        <v>6637.82</v>
+      </c>
+      <c r="C64" s="18" t="n">
+        <v>4425.21</v>
+      </c>
+      <c r="D64" s="18" t="n">
+        <v>6267.5</v>
+      </c>
+      <c r="E64" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="35" t="n">
+        <v>17330.53</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2406 Premier Custom Homes Quote</t>
+        </is>
+      </c>
+      <c r="B65" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C65" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="18" t="n">
+        <v>17262.74</v>
+      </c>
+      <c r="F65" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="35" t="n">
+        <v>17262.74</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>2024.929 DEEM Warehouse</t>
+        </is>
+      </c>
+      <c r="B66" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C66" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="18" t="n">
+        <v>15645.5</v>
+      </c>
+      <c r="E66" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="35" t="n">
+        <v>15645.5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>2025.1021 Convivio</t>
+        </is>
+      </c>
+      <c r="B67" s="18" t="n">
+        <v>2250</v>
+      </c>
+      <c r="C67" s="18" t="n">
+        <v>12458.26</v>
+      </c>
+      <c r="D67" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="35" t="n">
+        <v>14708.26</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2432 Liberty Assisted LIving 0528</t>
+        </is>
+      </c>
+      <c r="B68" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="18" t="n">
+        <v>12455.2</v>
+      </c>
+      <c r="G68" s="35" t="n">
+        <v>12455.2</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2380 Mike Valentine 0129</t>
+        </is>
+      </c>
+      <c r="B69" s="18" t="n">
+        <v>12430.13</v>
+      </c>
+      <c r="C69" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="35" t="n">
+        <v>12430.13</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2365 GSI Sackstedor Bloomington</t>
+        </is>
+      </c>
+      <c r="B70" s="18" t="n">
+        <v>11604.16</v>
+      </c>
+      <c r="C70" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="35" t="n">
+        <v>11604.16</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2401 Flores Kenneland</t>
+        </is>
+      </c>
+      <c r="B71" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C71" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="18" t="n">
+        <v>11454.33</v>
+      </c>
+      <c r="E71" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="35" t="n">
+        <v>11454.33</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>2026.1040 Lakeside Books</t>
+        </is>
+      </c>
+      <c r="B72" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C72" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="18" t="n">
+        <v>10020</v>
+      </c>
+      <c r="G72" s="35" t="n">
+        <v>10020</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2412 10732 Heaven Cove Way</t>
+        </is>
+      </c>
+      <c r="B73" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C73" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="18" t="n">
+        <v>10008.15</v>
+      </c>
+      <c r="G73" s="35" t="n">
+        <v>10008.15</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>2025.1031 Pita Way</t>
+        </is>
+      </c>
+      <c r="B74" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" s="18" t="n">
+        <v>8770.5</v>
+      </c>
+      <c r="D74" s="18" t="n">
+        <v>974.5</v>
+      </c>
+      <c r="E74" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="35" t="n">
+        <v>9745</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2433 Liberty Assisted Living 0529</t>
+        </is>
+      </c>
+      <c r="B75" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C75" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="18" t="n">
+        <v>9607.6</v>
+      </c>
+      <c r="G75" s="35" t="n">
+        <v>9607.6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>2025.984 Whiteland Indiana Guard Shack</t>
+        </is>
+      </c>
+      <c r="B76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="18" t="n">
+        <v>9200</v>
+      </c>
+      <c r="G76" s="35" t="n">
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2375 1802 Alabama St</t>
+        </is>
+      </c>
+      <c r="B77" s="18" t="n">
+        <v>9073.559999999999</v>
+      </c>
+      <c r="C77" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="35" t="n">
+        <v>9073.559999999999</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2389 Courtyards of Russell Oaks 145</t>
+        </is>
+      </c>
+      <c r="B78" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C78" s="18" t="n">
+        <v>8375.35</v>
+      </c>
+      <c r="D78" s="18" t="n">
+        <v>299.6</v>
+      </c>
+      <c r="E78" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="35" t="n">
+        <v>8674.950000000001</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2421 Flores Ohio Job</t>
+        </is>
+      </c>
+      <c r="B79" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C79" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="18" t="n">
+        <v>8624.08</v>
+      </c>
+      <c r="G79" s="35" t="n">
+        <v>8624.08</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2394 5778 Marvie Drive</t>
+        </is>
+      </c>
+      <c r="B80" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" s="18" t="n">
+        <v>8586.040000000001</v>
+      </c>
+      <c r="D80" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="35" t="n">
+        <v>8586.040000000001</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2392 3705 Holiday Farms Blvd - Precision</t>
+        </is>
+      </c>
+      <c r="B81" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" s="18" t="n">
+        <v>8393.530000000001</v>
+      </c>
+      <c r="D81" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="35" t="n">
+        <v>8393.530000000001</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2383 Courtyards of Cielo Ranch 37</t>
+        </is>
+      </c>
+      <c r="B82" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" s="18" t="n">
+        <v>7718.84</v>
+      </c>
+      <c r="D82" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="35" t="n">
+        <v>7718.84</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2363 Courtyards of Westfield 96</t>
+        </is>
+      </c>
+      <c r="B83" s="18" t="n">
+        <v>7700.52</v>
+      </c>
+      <c r="C83" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="35" t="n">
+        <v>7700.52</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2400 Courtyards of Russell Oaks 115</t>
+        </is>
+      </c>
+      <c r="B84" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="18" t="n">
+        <v>7645.75</v>
+      </c>
+      <c r="E84" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="35" t="n">
+        <v>7645.75</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2378 Courtyards of Westfield 108</t>
+        </is>
+      </c>
+      <c r="B85" s="18" t="n">
+        <v>7637.37</v>
+      </c>
+      <c r="C85" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="35" t="n">
+        <v>7637.37</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2410 Courtyards of Russell Oaks 113</t>
+        </is>
+      </c>
+      <c r="B86" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="18" t="n">
+        <v>7585.02</v>
+      </c>
+      <c r="F86" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="35" t="n">
+        <v>7585.02</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2369 Courtyards of Westfield 111</t>
+        </is>
+      </c>
+      <c r="B87" s="18" t="n">
+        <v>7574.01</v>
+      </c>
+      <c r="C87" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="35" t="n">
+        <v>7574.01</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2377 Courtyards of Cielo Ranch 38</t>
+        </is>
+      </c>
+      <c r="B88" s="18" t="n">
+        <v>7574.01</v>
+      </c>
+      <c r="C88" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="35" t="n">
+        <v>7574.01</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2402 Courtyards of Cielo Ranch 17</t>
+        </is>
+      </c>
+      <c r="B89" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C89" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="18" t="n">
+        <v>7307.29</v>
+      </c>
+      <c r="E89" s="18" t="n">
+        <v>240.36</v>
+      </c>
+      <c r="F89" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="35" t="n">
+        <v>7547.65</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2398 Courtyards of Ceilo Ranch 26</t>
+        </is>
+      </c>
+      <c r="B90" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" s="18" t="n">
+        <v>7276.63</v>
+      </c>
+      <c r="E90" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="35" t="n">
+        <v>7276.63</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2368 Courtyards of Russell Oaks 60</t>
+        </is>
+      </c>
+      <c r="B91" s="18" t="n">
+        <v>7243.75</v>
+      </c>
+      <c r="C91" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="35" t="n">
+        <v>7243.75</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2405 21569 Anchor Bay Drive</t>
+        </is>
+      </c>
+      <c r="B92" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E92" s="18" t="n">
+        <v>7033.52</v>
+      </c>
+      <c r="F92" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="35" t="n">
+        <v>7033.52</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2408 Courtyards of Westfield 107</t>
+        </is>
+      </c>
+      <c r="B93" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" s="18" t="n">
+        <v>6956.92</v>
+      </c>
+      <c r="F93" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="35" t="n">
+        <v>6956.92</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2385 Courtyards of Russell Oaks 123</t>
+        </is>
+      </c>
+      <c r="B94" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" s="18" t="n">
+        <v>6812.24</v>
+      </c>
+      <c r="D94" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" s="35" t="n">
+        <v>6812.24</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2371 13429 E 116th St</t>
+        </is>
+      </c>
+      <c r="B95" s="18" t="n">
+        <v>6806.08</v>
+      </c>
+      <c r="C95" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D95" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" s="35" t="n">
+        <v>6806.08</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>2026.1039 Upland Prospect Street</t>
+        </is>
+      </c>
+      <c r="B96" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" s="18" t="n">
+        <v>6500</v>
+      </c>
+      <c r="D96" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="35" t="n">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2386 Courtyards of Russell Oaks 125</t>
+        </is>
+      </c>
+      <c r="B97" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" s="18" t="n">
+        <v>6318.06</v>
+      </c>
+      <c r="D97" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E97" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" s="35" t="n">
+        <v>6318.06</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2388 Courtyards of Cielo Ranch 13</t>
+        </is>
+      </c>
+      <c r="B98" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" s="18" t="n">
+        <v>6290.19</v>
+      </c>
+      <c r="D98" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" s="35" t="n">
+        <v>6290.19</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2396 6252 West Turtle Hill Ct</t>
+        </is>
+      </c>
+      <c r="B99" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D99" s="18" t="n">
+        <v>6268.5</v>
+      </c>
+      <c r="E99" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F99" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="35" t="n">
+        <v>6268.5</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>2025.983 DEEM Warehouse Drop Ceiling</t>
+        </is>
+      </c>
+      <c r="B100" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C100" s="18" t="n">
+        <v>6200</v>
+      </c>
+      <c r="D100" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F100" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" s="35" t="n">
+        <v>6200</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2399 Courtyards of Russell Oaks 74</t>
+        </is>
+      </c>
+      <c r="B101" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C101" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D101" s="18" t="n">
+        <v>6156.42</v>
+      </c>
+      <c r="E101" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F101" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" s="35" t="n">
+        <v>6156.42</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2366 Courtyards of Cielo Ranch 15</t>
+        </is>
+      </c>
+      <c r="B102" s="18" t="n">
+        <v>6022.94</v>
+      </c>
+      <c r="C102" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D102" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" s="35" t="n">
+        <v>6022.94</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2370 Courtyards of Westfield 106</t>
+        </is>
+      </c>
+      <c r="B103" s="18" t="n">
+        <v>5971.55</v>
+      </c>
+      <c r="C103" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D103" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E103" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" s="35" t="n">
+        <v>5971.55</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2407 Courtyards of Russel Oaks 126</t>
+        </is>
+      </c>
+      <c r="B104" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C104" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" s="18" t="n">
+        <v>5928.42</v>
+      </c>
+      <c r="F104" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" s="35" t="n">
+        <v>5928.42</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2418 118 Centre Place</t>
+        </is>
+      </c>
+      <c r="B105" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C105" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" s="18" t="n">
+        <v>5520.75</v>
+      </c>
+      <c r="G105" s="35" t="n">
+        <v>5520.75</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2416 52 Centre Place</t>
+        </is>
+      </c>
+      <c r="B106" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C106" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" s="18" t="n">
+        <v>5520.75</v>
+      </c>
+      <c r="G106" s="35" t="n">
+        <v>5520.75</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2425 14 Parks</t>
+        </is>
+      </c>
+      <c r="B107" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C107" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" s="18" t="n">
+        <v>5520.75</v>
+      </c>
+      <c r="G107" s="35" t="n">
+        <v>5520.75</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2426 121 Centre Place</t>
+        </is>
+      </c>
+      <c r="B108" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C108" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" s="18" t="n">
+        <v>5520.75</v>
+      </c>
+      <c r="G108" s="35" t="n">
+        <v>5520.75</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2403 Big Dawg Pickup 0327</t>
+        </is>
+      </c>
+      <c r="B109" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C109" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" s="18" t="n">
+        <v>5302.49</v>
+      </c>
+      <c r="E109" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" s="35" t="n">
+        <v>5302.49</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2428 9 Centre Place</t>
+        </is>
+      </c>
+      <c r="B110" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C110" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" s="18" t="n">
+        <v>4962.27</v>
+      </c>
+      <c r="G110" s="35" t="n">
+        <v>4962.27</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2420 7508 Central Ave</t>
+        </is>
+      </c>
+      <c r="B111" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C111" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" s="18" t="n">
+        <v>4323.31</v>
+      </c>
+      <c r="G111" s="35" t="n">
+        <v>4323.31</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2384 225 N St Ave</t>
+        </is>
+      </c>
+      <c r="B112" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C112" s="18" t="n">
+        <v>4271.93</v>
+      </c>
+      <c r="D112" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" s="35" t="n">
+        <v>4271.93</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2417 117 Centre Place</t>
+        </is>
+      </c>
+      <c r="B113" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C113" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E113" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" s="18" t="n">
+        <v>4070.62</v>
+      </c>
+      <c r="G113" s="35" t="n">
+        <v>4070.62</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2419 120 Centre Place</t>
+        </is>
+      </c>
+      <c r="B114" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C114" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E114" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" s="18" t="n">
+        <v>4070.62</v>
+      </c>
+      <c r="G114" s="35" t="n">
+        <v>4070.62</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2372 Big Dawg Pickup 0115</t>
+        </is>
+      </c>
+      <c r="B115" s="18" t="n">
+        <v>3907.73</v>
+      </c>
+      <c r="C115" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" s="35" t="n">
+        <v>3907.73</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2424 10566 Coppergate</t>
+        </is>
+      </c>
+      <c r="B116" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C116" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" s="18" t="n">
+        <v>3882.79</v>
+      </c>
+      <c r="G116" s="35" t="n">
+        <v>3882.79</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2411 Clark Remodel</t>
+        </is>
+      </c>
+      <c r="B117" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C117" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" s="18" t="n">
+        <v>3764.86</v>
+      </c>
+      <c r="F117" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" s="35" t="n">
+        <v>3764.86</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2364 GSI 1-6</t>
+        </is>
+      </c>
+      <c r="B118" s="18" t="n">
+        <v>3762.61</v>
+      </c>
+      <c r="C118" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E118" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F118" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" s="35" t="n">
+        <v>3762.61</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2429 108 Centre Place</t>
+        </is>
+      </c>
+      <c r="B119" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C119" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E119" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F119" s="18" t="n">
+        <v>3711.4</v>
+      </c>
+      <c r="G119" s="35" t="n">
+        <v>3711.4</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2430 119 Centre Place</t>
+        </is>
+      </c>
+      <c r="B120" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C120" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D120" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E120" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" s="18" t="n">
+        <v>3411.3</v>
+      </c>
+      <c r="G120" s="35" t="n">
+        <v>3411.3</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2431 123 Centre Place</t>
+        </is>
+      </c>
+      <c r="B121" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C121" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D121" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E121" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" s="18" t="n">
+        <v>3411.3</v>
+      </c>
+      <c r="G121" s="35" t="n">
+        <v>3411.3</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2379 124 S A Street</t>
+        </is>
+      </c>
+      <c r="B122" s="18" t="n">
+        <v>2632.63</v>
+      </c>
+      <c r="C122" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D122" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E122" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F122" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" s="35" t="n">
+        <v>2632.63</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2414 10824 McPherson St</t>
+        </is>
+      </c>
+      <c r="B123" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C123" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E123" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F123" s="18" t="n">
+        <v>2611.31</v>
+      </c>
+      <c r="G123" s="35" t="n">
+        <v>2611.31</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2415 10826 McPherson St</t>
+        </is>
+      </c>
+      <c r="B124" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C124" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F124" s="18" t="n">
+        <v>2611.31</v>
+      </c>
+      <c r="G124" s="35" t="n">
+        <v>2611.31</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2423 10816 McPherson St</t>
+        </is>
+      </c>
+      <c r="B125" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C125" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E125" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" s="18" t="n">
+        <v>2611.31</v>
+      </c>
+      <c r="G125" s="35" t="n">
+        <v>2611.31</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2422 10814 McPherson St</t>
+        </is>
+      </c>
+      <c r="B126" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C126" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E126" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" s="18" t="n">
+        <v>2611.31</v>
+      </c>
+      <c r="G126" s="35" t="n">
+        <v>2611.31</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2390 510 W Pine St</t>
+        </is>
+      </c>
+      <c r="B127" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C127" s="18" t="n">
+        <v>2495.07</v>
+      </c>
+      <c r="D127" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G127" s="35" t="n">
+        <v>2495.07</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2391 0218 Jose Iracheta</t>
+        </is>
+      </c>
+      <c r="B128" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C128" s="18" t="n">
+        <v>2072.89</v>
+      </c>
+      <c r="D128" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F128" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" s="35" t="n">
+        <v>2072.89</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2427 Dapp Garage</t>
+        </is>
+      </c>
+      <c r="B129" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C129" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" s="18" t="n">
+        <v>2024.87</v>
+      </c>
+      <c r="G129" s="35" t="n">
+        <v>2024.87</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="13" t="inlineStr">
+        <is>
+          <t>2024.912 Upland Columbus</t>
+        </is>
+      </c>
+      <c r="B130" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C130" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" s="18" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G130" s="35" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="13" t="inlineStr">
+        <is>
+          <t>2025.999 Romet PWSI</t>
+        </is>
+      </c>
+      <c r="B131" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C131" s="18" t="n">
+        <v>1940</v>
+      </c>
+      <c r="D131" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" s="35" t="n">
+        <v>1940</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2381 Hunt Addition</t>
+        </is>
+      </c>
+      <c r="B132" s="18" t="n">
+        <v>1601.79</v>
+      </c>
+      <c r="C132" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" s="35" t="n">
+        <v>1601.79</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2374 Precision Pickup 0127</t>
+        </is>
+      </c>
+      <c r="B133" s="18" t="n">
+        <v>1151.37</v>
+      </c>
+      <c r="C133" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F133" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" s="35" t="n">
+        <v>1151.37</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2413 Precision Pickup 0501</t>
+        </is>
+      </c>
+      <c r="B134" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C134" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F134" s="18" t="n">
+        <v>1096.76</v>
+      </c>
+      <c r="G134" s="35" t="n">
+        <v>1096.76</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2382 Cohoat House</t>
+        </is>
+      </c>
+      <c r="B135" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C135" s="18" t="n">
+        <v>1065.45</v>
+      </c>
+      <c r="D135" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F135" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G135" s="35" t="n">
+        <v>1065.45</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2367 Courtyards of Russell Oaks 126</t>
+        </is>
+      </c>
+      <c r="B136" s="18" t="n">
+        <v>360.55</v>
+      </c>
+      <c r="C136" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" s="35" t="n">
+        <v>360.55</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2397 Courtyards of Cielo Ranch 26</t>
+        </is>
+      </c>
+      <c r="B137" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C137" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D137" s="18" t="n">
+        <v>360.55</v>
+      </c>
+      <c r="E137" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" s="35" t="n">
+        <v>360.55</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2362 Courtyards of Russel Oaks 127</t>
+        </is>
+      </c>
+      <c r="B138" s="18" t="n">
+        <v>299.6</v>
+      </c>
+      <c r="C138" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D138" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" s="35" t="n">
+        <v>299.6</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2395 Courtyards of Westfield 103</t>
+        </is>
+      </c>
+      <c r="B139" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C139" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D139" s="18" t="n">
+        <v>270.41</v>
+      </c>
+      <c r="E139" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" s="35" t="n">
+        <v>270.41</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2393 Precision Pickup 0216</t>
+        </is>
+      </c>
+      <c r="B140" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C140" s="18" t="n">
+        <v>252.01</v>
+      </c>
+      <c r="D140" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" s="35" t="n">
+        <v>252.01</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2373 Precision Pickup 0120</t>
+        </is>
+      </c>
+      <c r="B141" s="18" t="n">
+        <v>167.78</v>
+      </c>
+      <c r="C141" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" s="35" t="n">
+        <v>167.78</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="13" t="inlineStr">
+        <is>
+          <t>DS.2026.2409 Precision Pickup 0410</t>
+        </is>
+      </c>
+      <c r="B142" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C142" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" s="18" t="n">
+        <v>107.86</v>
+      </c>
+      <c r="F142" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" s="35" t="n">
+        <v>107.86</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="13" t="inlineStr">
+        <is>
+          <t>2024.874 Noblesville HS Academic Addition &amp; Renovation</t>
+        </is>
+      </c>
+      <c r="B143" s="18" t="n">
+        <v>-14964</v>
+      </c>
+      <c r="C143" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" s="35" t="n">
+        <v>-14964</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="13" t="inlineStr">
+        <is>
+          <t>MF.2024.875 Purdue Student Housing</t>
+        </is>
+      </c>
+      <c r="B144" s="18" t="n">
+        <v>-40103.3</v>
+      </c>
+      <c r="C144" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D144" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F144" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" s="35" t="n">
+        <v>-40103.3</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="36" t="inlineStr">
+        <is>
+          <t>TOTAL — all jobs</t>
+        </is>
+      </c>
+      <c r="B145" s="25" t="n">
+        <v>2479001.91</v>
+      </c>
+      <c r="C145" s="25" t="n">
+        <v>3525424.88</v>
+      </c>
+      <c r="D145" s="25" t="n">
+        <v>4583415.25</v>
+      </c>
+      <c r="E145" s="25" t="n">
+        <v>4672034.07</v>
+      </c>
+      <c r="F145" s="25" t="n">
+        <v>5022777.27</v>
+      </c>
+      <c r="G145" s="25" t="n">
+        <v>20282653.38</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G5:G144">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="004F98A3"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Source liquidity ratios from QuickBooks' own current/long-term classification
Fact_Cash now carries QB's CurrentAssets / CurrentLiabilities (from the balance
sheet summary breakdown). The workbook's Current ratio, Quick ratio, and Working
capital reference those instead of a re-derived split, so they match QuickBooks
exactly every refresh: current ratio 1.42 and working capital $5,789,885 == QB.

https://claude.ai/code/session_01CqWT8xJUtGR2BEPYF4o2h5
</commit_message>
<xml_diff>
--- a/mdg-powerbi/output/MDG_Executive_Dashboard.xlsx
+++ b/mdg-powerbi/output/MDG_Executive_Dashboard.xlsx
@@ -690,9 +690,9 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tCash" displayName="tCash" ref="A813:K814" headerRowCount="1">
-  <autoFilter ref="A813:K814"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tCash" displayName="tCash" ref="A813:M814" headerRowCount="1">
+  <autoFilter ref="A813:M814"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="CashBalance"/>
     <tableColumn id="3" name="LOCDrawn"/>
@@ -704,6 +704,8 @@
     <tableColumn id="9" name="LOCLimit"/>
     <tableColumn id="10" name="AdvanceRate"/>
     <tableColumn id="11" name="EligibleAR"/>
+    <tableColumn id="12" name="CurrentAssets"/>
+    <tableColumn id="13" name="CurrentLiabilities"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -1461,7 +1463,7 @@
       </c>
       <c r="D23" s="11" t="n"/>
       <c r="E23" s="26">
-        <f>IFERROR((SUMIFS(tBS[Amount],tBS[Section],"Assets")-SUMIFS(tBS[Amount],tBS[Account],"Fixed Assets")-SUMIFS(tBS[Amount],tBS[Account],"Other Assets"))/(SUMIFS(tBS[Amount],tBS[Section],"Liabilities")-SUMIFS(tBS[Amount],tBS[Account],"Long-term Liabilities")),0)</f>
+        <f>IFERROR(SUM(tCash[CurrentAssets])/SUM(tCash[CurrentLiabilities]),0)</f>
         <v/>
       </c>
       <c r="F23" s="11" t="n"/>
@@ -2114,7 +2116,7 @@
         </is>
       </c>
       <c r="B29" s="42">
-        <f>IFERROR((SUMIFS(tBS[Amount],tBS[Section],"Assets")-SUMIFS(tBS[Amount],tBS[Account],"Fixed Assets")-SUMIFS(tBS[Amount],tBS[Account],"Other Assets"))/(SUMIFS(tBS[Amount],tBS[Section],"Liabilities")-SUMIFS(tBS[Amount],tBS[Account],"Long-term Liabilities")),0)</f>
+        <f>IFERROR(SUM(tCash[CurrentAssets])/SUM(tCash[CurrentLiabilities]),0)</f>
         <v/>
       </c>
     </row>
@@ -2125,7 +2127,7 @@
         </is>
       </c>
       <c r="B30" s="42">
-        <f>IFERROR(((SUMIFS(tBS[Amount],tBS[Section],"Assets")-SUMIFS(tBS[Amount],tBS[Account],"Fixed Assets")-SUMIFS(tBS[Amount],tBS[Account],"Other Assets"))-SUMIFS(tBS[Amount],tBS[Account],"Drywall Inventory"))/(SUMIFS(tBS[Amount],tBS[Section],"Liabilities")-SUMIFS(tBS[Amount],tBS[Account],"Long-term Liabilities")),0)</f>
+        <f>IFERROR((SUM(tCash[CurrentAssets])-SUMIFS(tBS[Amount],tBS[Account],"Drywall Inventory"))/SUM(tCash[CurrentLiabilities]),0)</f>
         <v/>
       </c>
     </row>
@@ -2136,7 +2138,7 @@
         </is>
       </c>
       <c r="B31" s="36">
-        <f>(SUMIFS(tBS[Amount],tBS[Section],"Assets")-SUMIFS(tBS[Amount],tBS[Account],"Fixed Assets")-SUMIFS(tBS[Amount],tBS[Account],"Other Assets"))-(SUMIFS(tBS[Amount],tBS[Section],"Liabilities")-SUMIFS(tBS[Amount],tBS[Account],"Long-term Liabilities"))</f>
+        <f>SUM(tCash[CurrentAssets])-SUM(tCash[CurrentLiabilities])</f>
         <v/>
       </c>
     </row>
@@ -54094,6 +54096,16 @@
           <t>EligibleAR</t>
         </is>
       </c>
+      <c r="L813" s="54" t="inlineStr">
+        <is>
+          <t>CurrentAssets</t>
+        </is>
+      </c>
+      <c r="M813" s="54" t="inlineStr">
+        <is>
+          <t>CurrentLiabilities</t>
+        </is>
+      </c>
     </row>
     <row r="814">
       <c r="A814" s="55" t="inlineStr">
@@ -54130,6 +54142,12 @@
       </c>
       <c r="K814" s="56" t="n">
         <v>12986875.87</v>
+      </c>
+      <c r="L814" s="56" t="n">
+        <v>19633898.04</v>
+      </c>
+      <c r="M814" s="56" t="n">
+        <v>13844013.44</v>
       </c>
     </row>
     <row r="816">

</xml_diff>